<commit_message>
Implement 3D Ray-Tracer for Reverse Responder and reordered React navigation UI
</commit_message>
<xml_diff>
--- a/Radiation_Safety_Core_Documents.xlsx
+++ b/Radiation_Safety_Core_Documents.xlsx
@@ -10,7 +10,7 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="8_{AA835B7E-263F-47C4-8B05-3E31CD9DF651}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28725" yWindow="-22005" windowWidth="51840" windowHeight="21120" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView minimized="1" xWindow="5483" yWindow="1267" windowWidth="16200" windowHeight="9316" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Claude Log" sheetId="9" r:id="rId1"/>
@@ -6332,7 +6332,7 @@
 
 <file path=xl/webextensions/taskpanes.xml><?xml version="1.0" encoding="utf-8"?>
 <wetp:taskpanes xmlns:wetp="http://schemas.microsoft.com/office/webextensions/taskpanes/2010/11">
-  <wetp:taskpane dockstate="right" visibility="0" width="350" row="1">
+  <wetp:taskpane dockstate="right" visibility="0" width="700" row="1">
     <wetp:webextensionref xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
   </wetp:taskpane>
 </wetp:taskpanes>

</xml_diff>